<commit_message>
fix: Improve technical specs extraction from IDML
- Add story-based specs extraction (specs stored as text, not XML tables)
- Parse vertical table format: Header, Value1, Value2, Header2...
- Add comprehensive Italian->English header mappings
- Fix Hz typo correction to avoid double-z issue
- Now extracting: voltage, power, weight, IP rating, temperature, etc.

Example extraction improvement:
- Before: 1 row with empty specs
- After: 2 rows with 746 C Z16/Z20, 220-240V~ 50/60 Hz, 150 W, IP44
</commit_message>
<xml_diff>
--- a/output/learning/090-091_400.xlsx
+++ b/output/learning/090-091_400.xlsx
@@ -527,28 +527,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="33" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -649,11 +649,221 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>altO</t>
-        </is>
-      </c>
+          <t>400 CBC</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>220-240V~ 50/60 Hz</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Asincrono monofase</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>220 W</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>8,6 Kg</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1034 x 85 x 119 mm</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>IP55</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>-20°C ÷ + 55°C</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>70 cicli/ora</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>10 mm/s (*)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>270 mm</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Non compresa</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>400 SB</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>10 Kg</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1277 x 85 x 119 mm</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>60 cicli/ora</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>7,5 mm/s (*)</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>390 mm</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>(*) dati riferiti a 230V~ 50Hz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>400 SBS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>70 cicli/ora</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>10 mm/s (*)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>400 CBAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>50 cicli/ora</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>15 mm/s (*)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>400 CBAC L</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>40 cicli/ora</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>7,5 mm/s (*)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>